<commit_message>
Update company name keys for リクルート KS: align difficulty table and Excel sheet names
- COMPANY_PASS_DIFFICULTY: ホットペッパービューティー→リクルート社（KS美容）, SUUMOカウンター→リクルート社（SUUMOカウンター）
- Excel: update company names and Must要件 for both KS sheets

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/求人確度出力マスターシート.xlsx
+++ b/求人確度出力マスターシート.xlsx
@@ -2409,7 +2409,7 @@
     <row r="1" ht="30" customHeight="1" s="33">
       <c r="A1" s="36" t="inlineStr">
         <is>
-          <t>求人票データ｜株式会社リクルート（飲食・ビューティー領域 KS）</t>
+          <t>求人票データ▶▶リクルート社（KS美容）</t>
         </is>
       </c>
       <c r="B1" s="35" t="n"/>
@@ -2430,10 +2430,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>・自ら考え、自ら動くことができる方
-・常に学ぶ姿勢があり、成長したい意志がある方
-・カスタマーに新しい行動を生み出す「きっかけ」を創りたい方
-※約6割が営業職未経験からの入社</t>
+          <t>未経験可（社会人経験不問）/ 自走力・成長意欲のある方 / 顧客折衝・接客・対話経験があれば尚可 / ※契約社員スタート（正社員登用制度あり・年2回）</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3120,7 @@
     <row r="1" ht="30" customHeight="1" s="33">
       <c r="A1" s="36" t="inlineStr">
         <is>
-          <t>求人票データ｜株式会社リクルート_SUUMOカウンター領域</t>
+          <t>求人票データ▶▶リクルート社（SUUMOカウンター）</t>
         </is>
       </c>
       <c r="B1" s="35" t="n"/>
@@ -3144,12 +3141,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>・会話のキャッチボールが的確にできる方
-・他者に対する貢献にやりがいや喜びを感じられる方
-・周囲と協力しながら、チームで仕事に取り組む姿勢のある方
-・周囲からのアドバイスを素直に受け止め改善することができる方
-・分からないことや不安なことを自己開示し周囲を頼ることができる方
-※住宅業界知識不問（メンバーの8割が未経験入社）</t>
+          <t>未経験可 / ヒアリング・対話力のある方 / 土日祝メイン勤務可能な方 / 顧客に寄り添い伴走できる方</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unify company names across Excel and difficulty table (57 companies)
Excel:
- Add ▶▶ labels to BuySell(店舗/フィールド) and セレブリックス(チャネル戦略) sheets
- Fix 15 entries in 候補者一覧: XMile, BREXA, ウィルオブ, リクルートKS×6, ソフトバンク, IDOM, UZUZ, SUUMOカウンター×2

app.py COMPANY_PASS_DIFFICULTY:
- Add アシュアード(H=2), ブレクサテクノロジー/大東建託/ボードルア/オープンハウス(H=3)
- Rename ミガロホールディングス → プロパティエージェント(H=4)
- All 57 companies now have registered H values

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/求人確度出力マスターシート.xlsx
+++ b/求人確度出力マスターシート.xlsx
@@ -1094,7 +1094,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>XMile株式会社</t>
+          <t>エックスマイル</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>株式会社BREXA Technology（旧株式会社アウトソーシングテクノロジー）</t>
+          <t>ブレクサテクノロジー</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>株式会社ウィルオブ・コンストラクション</t>
+          <t>ウィルオブコンストラクション</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>株式会社リクルート_飲食・ビューティー領域（KS）</t>
+          <t>リクルート社（KS美容）</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ソフトバンク株式会社</t>
+          <t>ソフトバンク販売クルー</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>株式会社リクルート_SUUMOカウンター領域</t>
+          <t>リクルート社（SUUMOカウンター）</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>株式会社リクルート_飲食・ビューティー領域（KS）</t>
+          <t>リクルート社（KS美容）</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>株式会社リクルート_飲食・ビューティー領域（KS）</t>
+          <t>リクルート社（KS美容）</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>株式会社リクルート_住宅領域</t>
+          <t>リクルート社（SUUMOカウンター）</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>株式会社BREXA Technology（旧株式会社アウトソーシングテクノロジー）</t>
+          <t>ブレクサテクノロジー</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>株式会社IDOM</t>
+          <t>ガリバー</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>株式会社リクルート_飲食・ビューティー領域（KS）</t>
+          <t>リクルート社（KS美容）</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>株式会社UZUZ</t>
+          <t>ウズウズ</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>株式会社リクルート_飲食・ビューティー領域（KS）</t>
+          <t>リクルート社（KS美容）</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>株式会社リクルート_飲食・ビューティー領域（KS）</t>
+          <t>リクルート社（KS美容）</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>求人票データ｜株式会社BuySell Technologies（店舗事業本部）</t>
+          <t>求人票データ▶▶BuySell（店舗事業本部）</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>求人票データ｜株式会社BuySell Technologies（フィールドセールス事業本部）</t>
+          <t>求人票データ▶▶BuySell（フィールドセールス）</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>求人票データ｜株式会社セレブリックス セールスカンパニー（チャネル戦略事業本部）</t>
+          <t>求人票データ▶▶セレブリックス（チャネル戦略）</t>
         </is>
       </c>
     </row>

</xml_diff>